<commit_message>
Fix Pembrolizumab human data: replace incorrect de Vries 2023 survival plot with Shimizu 2016 PK data
Removed 15 rows sourced from de Vries 2023 Fig 3 (survival/follow-up plot, not PK).
Added 16 rows digitized from Shimizu 2016 Fig 1: 2 mg/kg (N=3) and 10 mg/kg (N=6-7)
serum concentration-time profiles, 8 timepoints each, 0-672 h.
Updated .gitignore to retain 2026-06-22 12-18 run. Removed stale AUC caveat note
from Script 03 that referenced the incorrect partial-AUC data.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Test2/03_Apriori/V2/Configurations/Applications.xlsx
+++ b/Test2/03_Apriori/V2/Configurations/Applications.xlsx
@@ -43,12 +43,13 @@
     <sheet name="Nivolumab_Human_20_mpk" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="Nivolumab_Monkey_1_mpk" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="Nivolumab_Monkey_10_mpk" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="Pembrolizumab_Human_3_mpk" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="Pembrolizumab_Monkey_0.3_mpk" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Pembrolizumab_Monkey_3_mpk" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="Pembrolizumab_Monkey_30_mpk" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="Tocilizumab_Human_8_mpk" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="Tocilizumab_Monkey_10_mpk" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Pembrolizumab_Human_2_mpk" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Pembrolizumab_Human_10_mpk" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Pembrolizumab_Monkey_0.3_mpk" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Pembrolizumab_Monkey_3_mpk" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Pembrolizumab_Monkey_30_mpk" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Tocilizumab_Human_8_mpk" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Tocilizumab_Monkey_10_mpk" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
 </workbook>
 </file>
@@ -2277,7 +2278,7 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -2336,6 +2337,124 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
         <v>0.3</v>
       </c>
       <c r="D2" t="s">
@@ -2354,124 +2473,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -2513,6 +2514,65 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
         <v>30</v>
       </c>
       <c r="D2" t="s">
@@ -2531,65 +2591,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="n">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
@@ -2631,6 +2632,65 @@
         <v>7</v>
       </c>
       <c r="C2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="55.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="8.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="18.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
         <v>10</v>
       </c>
       <c r="D2" t="s">

</xml_diff>